<commit_message>
good return  ENG add
</commit_message>
<xml_diff>
--- a/Form-Layout/ImportLayouts/Config/RPT_Import_Map.xlsx
+++ b/Form-Layout/ImportLayouts/Config/RPT_Import_Map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Film\GIT\SDA\Form-Layout\ImportLayouts\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEBB9EF-BBBF-41CE-9969-E878E9DA3996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44225D37-C5D0-4F50-9D1D-AD42B4BB0321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{014D90F8-196E-40BF-BFE8-06F39FDF4BE1}"/>
+    <workbookView xWindow="-6816" yWindow="-16512" windowWidth="23040" windowHeight="12120" xr2:uid="{014D90F8-196E-40BF-BFE8-06F39FDF4BE1}"/>
   </bookViews>
   <sheets>
     <sheet name="RPT_MAP" sheetId="1" r:id="rId1"/>

</xml_diff>